<commit_message>
tested ultrasensitivity. Fixed PPO (hopefully)
</commit_message>
<xml_diff>
--- a/apps_MAK_REINFORCE/RPA_3species_5rxns/RPA_3species_5rxns_MAK_REINFORCE.xlsx
+++ b/apps_MAK_REINFORCE/RPA_3species_5rxns/RPA_3species_5rxns_MAK_REINFORCE.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.14785714285714" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
@@ -483,6 +483,21 @@
           <t>2025-11-11 16:09:54</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2025-11-12 10:06:40</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>2025-11-13 09:17:45</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2025-11-13 09:19:02</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="17.25" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
@@ -505,6 +520,21 @@
           <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/4303dbd728384397adae5732c85f222a</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/be05dede1c0b4cabab460e35778d28f6</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/d9a2ac0ad6c140bf94e2e435a4a4ce8d</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/9851c5f84fc1458888fad7048195f741</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="19.5" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
@@ -521,6 +551,15 @@
       <c r="D3" t="n">
         <v>5</v>
       </c>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
@@ -537,6 +576,15 @@
       <c r="D4" t="n">
         <v>3</v>
       </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -553,6 +601,15 @@
       <c r="D5" t="n">
         <v>2</v>
       </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6" ht="19.5" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -569,6 +626,15 @@
       <c r="D6" t="n">
         <v>1280</v>
       </c>
+      <c r="E6" t="n">
+        <v>80</v>
+      </c>
+      <c r="F6" t="n">
+        <v>80</v>
+      </c>
+      <c r="G6" t="n">
+        <v>240</v>
+      </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -585,6 +651,15 @@
       <c r="D7" t="b">
         <v>0</v>
       </c>
+      <c r="E7" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -601,6 +676,15 @@
       <c r="D8" t="n">
         <v>0.0001</v>
       </c>
+      <c r="E8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
@@ -617,6 +701,15 @@
       <c r="D9" t="n">
         <v>300</v>
       </c>
+      <c r="E9" t="n">
+        <v>300</v>
+      </c>
+      <c r="F9" t="n">
+        <v>300</v>
+      </c>
+      <c r="G9" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="10" ht="19.5" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -633,6 +726,15 @@
       <c r="D10" t="n">
         <v>5</v>
       </c>
+      <c r="E10" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11" ht="19.5" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
@@ -649,6 +751,15 @@
       <c r="D11" t="n">
         <v>1024</v>
       </c>
+      <c r="E11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1024</v>
+      </c>
     </row>
     <row r="12" ht="19.5" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -665,6 +776,15 @@
       <c r="D12" t="n">
         <v>10240</v>
       </c>
+      <c r="E12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="F12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="G12" t="n">
+        <v>10240</v>
+      </c>
     </row>
     <row r="13" ht="19.5" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
@@ -681,6 +801,15 @@
       <c r="D13" t="n">
         <v>128</v>
       </c>
+      <c r="E13" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -703,6 +832,21 @@
           <t>{'entropy_weight': 0.001, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.001}</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.001, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.001}</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.001, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.001}</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.001, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.001}</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="17.25" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
@@ -725,6 +869,21 @@
           <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="19.5" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -741,6 +900,15 @@
       <c r="D16" t="n">
         <v>1</v>
       </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" ht="19.5" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
@@ -757,6 +925,15 @@
       <c r="D17" t="n">
         <v>10</v>
       </c>
+      <c r="E17" t="n">
+        <v>10</v>
+      </c>
+      <c r="F17" t="n">
+        <v>10</v>
+      </c>
+      <c r="G17" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
@@ -773,6 +950,15 @@
       <c r="D18" t="n">
         <v>200</v>
       </c>
+      <c r="E18" t="n">
+        <v>200</v>
+      </c>
+      <c r="F18" t="n">
+        <v>200</v>
+      </c>
+      <c r="G18" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
@@ -789,6 +975,15 @@
       <c r="D19" t="n">
         <v>1000</v>
       </c>
+      <c r="E19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1000</v>
+      </c>
     </row>
     <row r="20" ht="19.5" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
@@ -805,6 +1000,15 @@
       <c r="D20" t="n">
         <v>1</v>
       </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21" ht="19.5" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
@@ -821,6 +1025,15 @@
       <c r="D21" t="n">
         <v>9</v>
       </c>
+      <c r="E21" t="n">
+        <v>9</v>
+      </c>
+      <c r="F21" t="n">
+        <v>9</v>
+      </c>
+      <c r="G21" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="22" ht="17.25" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
@@ -839,6 +1052,21 @@
         </is>
       </c>
       <c r="D22" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
         <is>
           <t>{'type': 'lognormal_1D'}</t>
         </is>

</xml_diff>